<commit_message>
les programmes des classes en college(secondaire)
</commit_message>
<xml_diff>
--- a/resources/Programmes/Programmeclasse3ecollege.xlsx
+++ b/resources/Programmes/Programmeclasse3ecollege.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24527"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Documents\JANGAA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JEANNE\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CCA748FF-5ED4-42DB-8E1E-C71754FA9260}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7155"/>
   </bookViews>
   <sheets>
     <sheet name="Feuille 1" sheetId="1" r:id="rId1"/>
@@ -20,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="224">
   <si>
     <t>Matière</t>
   </si>
@@ -761,12 +760,15 @@
   <si>
     <t>1. Rédaction guidée
 2. Exercices de conjugaison</t>
+  </si>
+  <si>
+    <t>null</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -1053,12 +1055,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AA55"/>
+  <dimension ref="A1:AA43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="2" max="2" width="27.28515625" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" customWidth="1"/>
+    <col min="4" max="4" width="24.5703125" customWidth="1"/>
+    <col min="5" max="5" width="24.85546875" customWidth="1"/>
+    <col min="6" max="6" width="31.140625" customWidth="1"/>
+    <col min="7" max="7" width="22.140625" customWidth="1"/>
+    <col min="8" max="8" width="21.140625" customWidth="1"/>
+    <col min="9" max="9" width="17" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -1107,7 +1120,7 @@
       <c r="Z1" s="2"/>
       <c r="AA1" s="2"/>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:27" ht="57" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
@@ -1136,7 +1149,10 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:27" ht="71.25" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>223</v>
+      </c>
       <c r="B3" s="4" t="s">
         <v>18</v>
       </c>
@@ -1162,7 +1178,10 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:27" ht="57" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>223</v>
+      </c>
       <c r="B4" s="4" t="s">
         <v>23</v>
       </c>
@@ -1188,73 +1207,108 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
+    <row r="5" spans="1:27" ht="71.25" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
         <v>28</v>
       </c>
+      <c r="B5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" ht="57" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>223</v>
+      </c>
       <c r="B6" s="4" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>15</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="I6" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:27" ht="57" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>223</v>
+      </c>
       <c r="B7" s="4" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="G7" s="4" t="s">
         <v>15</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" ht="57" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>223</v>
+      </c>
       <c r="B8" s="4" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>15</v>
@@ -1263,203 +1317,317 @@
         <v>15</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="B9" s="4" t="s">
-        <v>47</v>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>54</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>15</v>
+        <v>58</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>52</v>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>223</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="11" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G11" s="4" t="s">
         <v>59</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="I11" s="4" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="12" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>223</v>
+      </c>
       <c r="B12" s="5" t="s">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
+        <v>76</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>223</v>
+      </c>
       <c r="H12" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="I12" s="6"/>
-    </row>
-    <row r="14" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>68</v>
+        <v>77</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27" ht="71.25" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27" ht="57" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>223</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>85</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>59</v>
+        <v>14</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="15" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="5" t="s">
-        <v>73</v>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" ht="57" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>223</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>90</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>74</v>
+        <v>91</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
+        <v>93</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>83</v>
+      </c>
       <c r="H15" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="I15" s="6"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A17" s="3" t="s">
-        <v>78</v>
+        <v>94</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27" ht="71.25" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>223</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="57" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>223</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>79</v>
+        <v>101</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>80</v>
+        <v>102</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>81</v>
+        <v>103</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>82</v>
+        <v>104</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>84</v>
+        <v>105</v>
       </c>
       <c r="I17" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" ht="42.75" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>223</v>
+      </c>
       <c r="B18" s="4" t="s">
-        <v>85</v>
+        <v>106</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>86</v>
+        <v>107</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>87</v>
+        <v>108</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>88</v>
+        <v>109</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>14</v>
+        <v>99</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>89</v>
+        <v>110</v>
       </c>
       <c r="I18" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" ht="42.75" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>223</v>
+      </c>
       <c r="B19" s="4" t="s">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>92</v>
+        <v>113</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>93</v>
+        <v>114</v>
       </c>
       <c r="F19" s="4" t="s">
         <v>15</v>
@@ -1468,24 +1636,27 @@
         <v>83</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>94</v>
+        <v>115</v>
       </c>
       <c r="I19" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9" ht="42.75" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>223</v>
+      </c>
       <c r="B20" s="4" t="s">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>96</v>
+        <v>117</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>97</v>
+        <v>118</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>98</v>
+        <v>119</v>
       </c>
       <c r="F20" s="4" t="s">
         <v>99</v>
@@ -1494,601 +1665,678 @@
         <v>99</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="I20" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B21" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>102</v>
+    <row r="21" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="B21" t="s">
+        <v>223</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>122</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>103</v>
+        <v>123</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>104</v>
+        <v>124</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>15</v>
+        <v>58</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>99</v>
+        <v>59</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>105</v>
+        <v>125</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B22" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>107</v>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>223</v>
+      </c>
+      <c r="B22" t="s">
+        <v>223</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>126</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>108</v>
+        <v>127</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="G22" s="4" t="s">
-        <v>99</v>
+        <v>128</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>223</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="I22" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B23" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>112</v>
+        <v>129</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="86.25" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>223</v>
+      </c>
+      <c r="B23" t="s">
+        <v>223</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>130</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>113</v>
+        <v>131</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="G23" s="4" t="s">
-        <v>83</v>
+        <v>132</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>223</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="I23" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B24" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>117</v>
+        <v>133</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="100.5" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B24" t="s">
+        <v>223</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>135</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>118</v>
+        <v>136</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>99</v>
+        <v>59</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>99</v>
+        <v>59</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>120</v>
+        <v>138</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>121</v>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="72" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>223</v>
+      </c>
+      <c r="B25" t="s">
+        <v>223</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="I25" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="72" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>223</v>
+      </c>
+      <c r="B26" t="s">
+        <v>223</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>122</v>
+        <v>143</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>123</v>
+        <v>144</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="F26" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="57.75" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>223</v>
+      </c>
+      <c r="B27" t="s">
+        <v>223</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="72" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>223</v>
+      </c>
+      <c r="B28" t="s">
+        <v>223</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="I28" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="43.5" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="F29" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="G29" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="H26" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="I26" s="4" t="s">
+      <c r="H29" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="I29" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C27" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
-      <c r="H27" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="I27" s="6"/>
-    </row>
-    <row r="28" spans="1:9" ht="143.25" x14ac:dyDescent="0.25">
-      <c r="C28" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="F28" s="6"/>
-      <c r="G28" s="6"/>
-      <c r="H28" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="I28" s="6"/>
-    </row>
-    <row r="30" spans="1:9" ht="100.5" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>135</v>
+    <row r="30" spans="1:9" ht="72" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>223</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>223</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>136</v>
+        <v>161</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="F30" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="I30" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="114.75" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F31" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="G30" s="4" t="s">
+      <c r="G31" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="H30" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="I30" s="4" t="s">
+      <c r="H31" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="I31" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="114.75" x14ac:dyDescent="0.25">
-      <c r="C31" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="F31" s="6"/>
-      <c r="G31" s="6"/>
-      <c r="H31" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="I31" s="6"/>
-    </row>
-    <row r="32" spans="1:9" ht="114.75" x14ac:dyDescent="0.25">
-      <c r="C32" s="5" t="s">
-        <v>143</v>
+    <row r="32" spans="1:9" ht="72" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>223</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>171</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>144</v>
+        <v>172</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="F32" s="6"/>
-      <c r="G32" s="6"/>
+        <v>173</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>223</v>
+      </c>
       <c r="H32" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="I32" s="6"/>
-    </row>
-    <row r="33" spans="1:9" ht="114.75" x14ac:dyDescent="0.25">
-      <c r="C33" s="5" t="s">
-        <v>147</v>
+        <v>174</v>
+      </c>
+      <c r="I32" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="72" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>223</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>176</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>148</v>
+        <v>177</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="F33" s="6"/>
-      <c r="G33" s="6"/>
+        <v>178</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>223</v>
+      </c>
       <c r="H33" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="I33" s="6"/>
+        <v>179</v>
+      </c>
+      <c r="I33" s="6" t="s">
+        <v>223</v>
+      </c>
     </row>
     <row r="34" spans="1:9" ht="114.75" x14ac:dyDescent="0.25">
-      <c r="C34" s="5" t="s">
-        <v>151</v>
+      <c r="A34" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>181</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>152</v>
+        <v>182</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="F34" s="6"/>
-      <c r="G34" s="6"/>
+        <v>183</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>59</v>
+      </c>
       <c r="H34" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="I34" s="6"/>
+        <v>184</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="86.25" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>223</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="G35" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="I35" s="6" t="s">
+        <v>223</v>
+      </c>
     </row>
     <row r="36" spans="1:9" ht="100.5" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="B36" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="C36" s="6"/>
+        <v>190</v>
+      </c>
+      <c r="B36" t="s">
+        <v>223</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>191</v>
+      </c>
       <c r="D36" s="4" t="s">
-        <v>157</v>
+        <v>192</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>158</v>
+        <v>193</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G36" s="4" t="s">
         <v>59</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>159</v>
+        <v>194</v>
       </c>
       <c r="I36" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="129" x14ac:dyDescent="0.25">
-      <c r="B37" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="C37" s="6"/>
+    <row r="37" spans="1:9" ht="86.25" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>223</v>
+      </c>
+      <c r="B37" t="s">
+        <v>223</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>195</v>
+      </c>
       <c r="D37" s="4" t="s">
-        <v>161</v>
+        <v>196</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="F37" s="6"/>
-      <c r="G37" s="6"/>
+        <v>197</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>223</v>
+      </c>
       <c r="H37" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="I37" s="6"/>
-    </row>
-    <row r="39" spans="1:9" ht="114.75" x14ac:dyDescent="0.25">
+        <v>198</v>
+      </c>
+      <c r="I37" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="86.25" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>223</v>
+      </c>
+      <c r="B38" t="s">
+        <v>223</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="G38" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="I38" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="100.5" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="B39" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>166</v>
+        <v>203</v>
+      </c>
+      <c r="B39" t="s">
+        <v>223</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>204</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>167</v>
+        <v>205</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>168</v>
+        <v>206</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G39" s="4" t="s">
         <v>59</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>169</v>
+        <v>207</v>
       </c>
       <c r="I39" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="114.75" x14ac:dyDescent="0.25">
-      <c r="B40" s="5" t="s">
+    <row r="40" spans="1:9" ht="72" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>223</v>
+      </c>
+      <c r="B40" t="s">
+        <v>223</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="F40" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="G40" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="H40" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="I40" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="57.75" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>223</v>
+      </c>
+      <c r="B41" t="s">
+        <v>223</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="G41" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="I41" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="100.5" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="B42" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C40" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="D40" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="E40" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="F40" s="6"/>
-      <c r="G40" s="6"/>
-      <c r="H40" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="I40" s="6"/>
-    </row>
-    <row r="41" spans="1:9" ht="114.75" x14ac:dyDescent="0.25">
-      <c r="B41" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="F41" s="6"/>
-      <c r="G41" s="6"/>
-      <c r="H41" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="I41" s="6"/>
-    </row>
-    <row r="43" spans="1:9" ht="114.75" x14ac:dyDescent="0.25">
-      <c r="A43" s="3" t="s">
-        <v>180</v>
+      <c r="C42" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="H42" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="I42" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="72" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>223</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>181</v>
+        <v>220</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>182</v>
+        <v>221</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="F43" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="G43" s="4" t="s">
-        <v>59</v>
+        <v>222</v>
+      </c>
+      <c r="F43" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="G43" s="6" t="s">
+        <v>223</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="I43" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" ht="114.75" x14ac:dyDescent="0.25">
-      <c r="B44" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="C44" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="D44" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="E44" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="F44" s="6"/>
-      <c r="G44" s="6"/>
-      <c r="H44" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="I44" s="6"/>
-    </row>
-    <row r="46" spans="1:9" ht="100.5" x14ac:dyDescent="0.25">
-      <c r="A46" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="C46" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="D46" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="E46" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="F46" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="G46" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="H46" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="I46" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" ht="129" x14ac:dyDescent="0.25">
-      <c r="C47" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="D47" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="E47" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="F47" s="6"/>
-      <c r="G47" s="6"/>
-      <c r="H47" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="I47" s="6"/>
-    </row>
-    <row r="48" spans="1:9" ht="114.75" x14ac:dyDescent="0.25">
-      <c r="C48" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="D48" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="E48" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="F48" s="6"/>
-      <c r="G48" s="6"/>
-      <c r="H48" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="I48" s="6"/>
-    </row>
-    <row r="50" spans="1:9" ht="100.5" x14ac:dyDescent="0.25">
-      <c r="A50" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="C50" s="5" t="s">
-        <v>204</v>
-      </c>
-      <c r="D50" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="E50" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="F50" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="G50" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="H50" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="I50" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" ht="114.75" x14ac:dyDescent="0.25">
-      <c r="C51" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="D51" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="E51" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="F51" s="6"/>
-      <c r="G51" s="6"/>
-      <c r="H51" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="I51" s="6"/>
-    </row>
-    <row r="52" spans="1:9" ht="86.25" x14ac:dyDescent="0.25">
-      <c r="C52" s="5" t="s">
-        <v>212</v>
-      </c>
-      <c r="D52" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="E52" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="F52" s="6"/>
-      <c r="G52" s="6"/>
-      <c r="H52" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="I52" s="6"/>
-    </row>
-    <row r="54" spans="1:9" ht="100.5" x14ac:dyDescent="0.25">
-      <c r="A54" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="B54" s="5" t="s">
-        <v>170</v>
-      </c>
-      <c r="C54" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="D54" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="E54" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="F54" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="G54" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="H54" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="I54" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" ht="114.75" x14ac:dyDescent="0.25">
-      <c r="B55" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="D55" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="E55" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="F55" s="6"/>
-      <c r="G55" s="6"/>
-      <c r="H55" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="I55" s="6"/>
+      <c r="I43" s="6" t="s">
+        <v>223</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
quelques modifications sur les programmes par defauts
</commit_message>
<xml_diff>
--- a/resources/Programmes/Programmeclasse3ecollege.xlsx
+++ b/resources/Programmes/Programmeclasse3ecollege.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JEANNE\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\gestionscolaire\resources\Programmes\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="226">
   <si>
     <t>Matière</t>
   </si>
@@ -763,13 +763,19 @@
   </si>
   <si>
     <t>null</t>
+  </si>
+  <si>
+    <t>heure_debut</t>
+  </si>
+  <si>
+    <t>heure_fin</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -804,6 +810,12 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -825,7 +837,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -840,6 +852,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1059,7 +1074,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AA43"/>
+  <dimension ref="A1:AC43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -1069,11 +1084,11 @@
     <col min="5" max="5" width="24.85546875" customWidth="1"/>
     <col min="6" max="6" width="31.140625" customWidth="1"/>
     <col min="7" max="7" width="22.140625" customWidth="1"/>
-    <col min="8" max="8" width="21.140625" customWidth="1"/>
-    <col min="9" max="9" width="17" customWidth="1"/>
+    <col min="8" max="10" width="21.140625" customWidth="1"/>
+    <col min="11" max="11" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1099,10 +1114,14 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
       <c r="L1" s="2"/>
       <c r="M1" s="2"/>
       <c r="N1" s="2"/>
@@ -1119,8 +1138,10 @@
       <c r="Y1" s="2"/>
       <c r="Z1" s="2"/>
       <c r="AA1" s="2"/>
-    </row>
-    <row r="2" spans="1:27" ht="57" x14ac:dyDescent="0.2">
+      <c r="AB1" s="2"/>
+      <c r="AC1" s="2"/>
+    </row>
+    <row r="2" spans="1:29" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
@@ -1146,10 +1167,16 @@
         <v>16</v>
       </c>
       <c r="I2" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K2" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:27" ht="71.25" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:29" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>223</v>
       </c>
@@ -1175,10 +1202,16 @@
         <v>22</v>
       </c>
       <c r="I3" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K3" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:27" ht="57" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:29" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>223</v>
       </c>
@@ -1204,10 +1237,16 @@
         <v>27</v>
       </c>
       <c r="I4" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K4" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:27" ht="71.25" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:29" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>28</v>
       </c>
@@ -1233,10 +1272,16 @@
         <v>34</v>
       </c>
       <c r="I5" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K5" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:27" ht="57" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:29" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>223</v>
       </c>
@@ -1262,10 +1307,16 @@
         <v>40</v>
       </c>
       <c r="I6" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K6" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:27" ht="57" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:29" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>223</v>
       </c>
@@ -1291,10 +1342,16 @@
         <v>45</v>
       </c>
       <c r="I7" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K7" s="4" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:27" ht="57" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:29" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>223</v>
       </c>
@@ -1320,10 +1377,16 @@
         <v>51</v>
       </c>
       <c r="I8" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K8" s="4" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>53</v>
       </c>
@@ -1349,10 +1412,16 @@
         <v>60</v>
       </c>
       <c r="I9" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K9" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>223</v>
       </c>
@@ -1377,11 +1446,17 @@
       <c r="H10" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I10" s="6" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I10" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="11" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>67</v>
       </c>
@@ -1407,10 +1482,16 @@
         <v>72</v>
       </c>
       <c r="I11" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K11" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>223</v>
       </c>
@@ -1435,11 +1516,17 @@
       <c r="H12" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="I12" s="6" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="13" spans="1:27" ht="71.25" x14ac:dyDescent="0.2">
+      <c r="I12" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="13" spans="1:29" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>78</v>
       </c>
@@ -1465,10 +1552,16 @@
         <v>84</v>
       </c>
       <c r="I13" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K13" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:27" ht="57" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:29" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>223</v>
       </c>
@@ -1494,10 +1587,16 @@
         <v>89</v>
       </c>
       <c r="I14" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K14" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:27" ht="57" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:29" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>223</v>
       </c>
@@ -1523,10 +1622,16 @@
         <v>94</v>
       </c>
       <c r="I15" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K15" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:27" ht="71.25" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:29" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>223</v>
       </c>
@@ -1552,10 +1657,16 @@
         <v>100</v>
       </c>
       <c r="I16" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K16" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="57" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>223</v>
       </c>
@@ -1581,10 +1692,16 @@
         <v>105</v>
       </c>
       <c r="I17" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K17" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="42.75" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>223</v>
       </c>
@@ -1610,10 +1727,16 @@
         <v>110</v>
       </c>
       <c r="I18" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K18" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="42.75" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>223</v>
       </c>
@@ -1639,10 +1762,16 @@
         <v>115</v>
       </c>
       <c r="I19" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J19" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K19" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="42.75" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>223</v>
       </c>
@@ -1668,10 +1797,16 @@
         <v>120</v>
       </c>
       <c r="I20" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K20" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>121</v>
       </c>
@@ -1697,10 +1832,16 @@
         <v>125</v>
       </c>
       <c r="I21" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K21" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>223</v>
       </c>
@@ -1725,11 +1866,17 @@
       <c r="H22" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="I22" s="6" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" ht="86.25" x14ac:dyDescent="0.25">
+      <c r="I22" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J22" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>223</v>
       </c>
@@ -1754,11 +1901,17 @@
       <c r="H23" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="I23" s="6" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" ht="100.5" x14ac:dyDescent="0.25">
+      <c r="I23" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J23" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K23" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>134</v>
       </c>
@@ -1784,10 +1937,16 @@
         <v>138</v>
       </c>
       <c r="I24" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J24" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K24" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="72" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>223</v>
       </c>
@@ -1812,11 +1971,17 @@
       <c r="H25" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="I25" s="6" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" ht="72" x14ac:dyDescent="0.25">
+      <c r="I25" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J25" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K25" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>223</v>
       </c>
@@ -1841,11 +2006,17 @@
       <c r="H26" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="I26" s="6" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" ht="57.75" x14ac:dyDescent="0.25">
+      <c r="I26" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J26" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K26" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>223</v>
       </c>
@@ -1870,11 +2041,17 @@
       <c r="H27" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="I27" s="6" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" ht="72" x14ac:dyDescent="0.25">
+      <c r="I27" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J27" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K27" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>223</v>
       </c>
@@ -1899,11 +2076,17 @@
       <c r="H28" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="I28" s="6" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" ht="43.5" x14ac:dyDescent="0.25">
+      <c r="I28" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J28" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K28" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>155</v>
       </c>
@@ -1929,10 +2112,16 @@
         <v>159</v>
       </c>
       <c r="I29" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J29" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K29" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="72" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>223</v>
       </c>
@@ -1957,11 +2146,17 @@
       <c r="H30" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="I30" s="6" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" ht="114.75" x14ac:dyDescent="0.25">
+      <c r="I30" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J30" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K30" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>164</v>
       </c>
@@ -1987,10 +2182,16 @@
         <v>169</v>
       </c>
       <c r="I31" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J31" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K31" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="72" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>223</v>
       </c>
@@ -2015,11 +2216,17 @@
       <c r="H32" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="I32" s="6" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" ht="72" x14ac:dyDescent="0.25">
+      <c r="I32" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J32" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K32" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>223</v>
       </c>
@@ -2044,11 +2251,17 @@
       <c r="H33" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="I33" s="6" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" ht="114.75" x14ac:dyDescent="0.25">
+      <c r="I33" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J33" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K33" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>180</v>
       </c>
@@ -2074,10 +2287,16 @@
         <v>184</v>
       </c>
       <c r="I34" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J34" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K34" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="86.25" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>223</v>
       </c>
@@ -2102,11 +2321,17 @@
       <c r="H35" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="I35" s="6" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" ht="100.5" x14ac:dyDescent="0.25">
+      <c r="I35" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J35" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K35" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>190</v>
       </c>
@@ -2132,10 +2357,16 @@
         <v>194</v>
       </c>
       <c r="I36" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J36" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K36" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="86.25" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>223</v>
       </c>
@@ -2160,11 +2391,17 @@
       <c r="H37" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="I37" s="6" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" ht="86.25" x14ac:dyDescent="0.25">
+      <c r="I37" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J37" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K37" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>223</v>
       </c>
@@ -2189,11 +2426,17 @@
       <c r="H38" s="4" t="s">
         <v>202</v>
       </c>
-      <c r="I38" s="6" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" ht="100.5" x14ac:dyDescent="0.25">
+      <c r="I38" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J38" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K38" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>203</v>
       </c>
@@ -2219,10 +2462,16 @@
         <v>207</v>
       </c>
       <c r="I39" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J39" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K39" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="72" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>223</v>
       </c>
@@ -2247,11 +2496,17 @@
       <c r="H40" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="I40" s="6" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" ht="57.75" x14ac:dyDescent="0.25">
+      <c r="I40" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J40" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K40" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="43.5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>223</v>
       </c>
@@ -2276,11 +2531,17 @@
       <c r="H41" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="I41" s="6" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" ht="100.5" x14ac:dyDescent="0.25">
+      <c r="I41" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J41" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K41" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>216</v>
       </c>
@@ -2306,10 +2567,16 @@
         <v>219</v>
       </c>
       <c r="I42" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J42" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K42" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="72" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" ht="57.75" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>223</v>
       </c>
@@ -2334,11 +2601,18 @@
       <c r="H43" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="I43" s="6" t="s">
+      <c r="I43" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="J43" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="K43" s="6" t="s">
         <v>223</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>